<commit_message>
bug fixes and consistancy refacor
</commit_message>
<xml_diff>
--- a/Attendance Tabloid.xlsx
+++ b/Attendance Tabloid.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="550" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="533" uniqueCount="50">
   <si>
     <t>Name</t>
   </si>
@@ -96,9 +96,6 @@
   </si>
   <si>
     <t>Bingham, Kenye'</t>
-  </si>
-  <si>
-    <t>Brown, Trinity</t>
   </si>
   <si>
     <t>Butler, Malachi</t>
@@ -218,7 +215,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC9DAF8"/>
+        <fgColor rgb="FFD0E0E3"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -611,7 +608,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q26"/>
+  <dimension ref="A1:Q25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="26.7109375" customWidth="1"/>
@@ -2328,77 +2325,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:17">
-      <c r="A26" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="B26" s="2">
-        <f>'Week 1'!G26</f>
-        <v>0</v>
-      </c>
-      <c r="C26" s="2">
-        <f>'Week 2'!G26</f>
-        <v>0</v>
-      </c>
-      <c r="D26" s="2">
-        <f>'Week 3'!G26</f>
-        <v>0</v>
-      </c>
-      <c r="E26" s="2">
-        <f>'Week 4'!G26</f>
-        <v>0</v>
-      </c>
-      <c r="F26" s="2">
-        <f>'Week 5'!G26</f>
-        <v>0</v>
-      </c>
-      <c r="G26" s="2">
-        <f>'Week 6'!G26</f>
-        <v>0</v>
-      </c>
-      <c r="H26" s="2">
-        <f>'Week 7'!G26</f>
-        <v>0</v>
-      </c>
-      <c r="I26" s="2">
-        <f>'Week 8'!G26</f>
-        <v>0</v>
-      </c>
-      <c r="J26" s="2">
-        <f>'Week 9'!G26</f>
-        <v>0</v>
-      </c>
-      <c r="K26" s="2">
-        <f>'Week 10'!G26</f>
-        <v>0</v>
-      </c>
-      <c r="L26" s="2">
-        <f>'Week 11'!G26</f>
-        <v>0</v>
-      </c>
-      <c r="M26" s="2">
-        <f>'Week 12'!G26</f>
-        <v>0</v>
-      </c>
-      <c r="N26" s="2">
-        <f>'Week 13'!G26</f>
-        <v>0</v>
-      </c>
-      <c r="O26" s="2">
-        <f>'Week 14'!G26</f>
-        <v>0</v>
-      </c>
-      <c r="P26" s="2">
-        <f>'Week 15'!G26</f>
-        <v>0</v>
-      </c>
-      <c r="Q26" s="2">
-        <f>SUM(B26:P26)</f>
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:P26">
+  <conditionalFormatting sqref="B2:P25">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>0</formula>
     </cfRule>
@@ -2419,7 +2347,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.140625" customWidth="1"/>
@@ -2432,25 +2360,25 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>48</v>
-      </c>
       <c r="G1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -2466,9 +2394,6 @@
       <c r="D2" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E2" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G2" s="4">
         <f>COUNTIF(B2:E2, TRUE)</f>
         <v>0</v>
@@ -2491,9 +2416,6 @@
       <c r="D3" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E3" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G3" s="4">
         <f>COUNTIF(B3:E3, TRUE)</f>
         <v>0</v>
@@ -2516,9 +2438,6 @@
       <c r="D4" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E4" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G4" s="4">
         <f>COUNTIF(B4:E4, TRUE)</f>
         <v>0</v>
@@ -2541,9 +2460,6 @@
       <c r="D5" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E5" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G5" s="4">
         <f>COUNTIF(B5:E5, TRUE)</f>
         <v>0</v>
@@ -2566,9 +2482,6 @@
       <c r="D6" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E6" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G6" s="4">
         <f>COUNTIF(B6:E6, TRUE)</f>
         <v>0</v>
@@ -2591,9 +2504,6 @@
       <c r="D7" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E7" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G7" s="4">
         <f>COUNTIF(B7:E7, TRUE)</f>
         <v>0</v>
@@ -2616,9 +2526,6 @@
       <c r="D8" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E8" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G8" s="4">
         <f>COUNTIF(B8:E8, TRUE)</f>
         <v>0</v>
@@ -2641,9 +2548,6 @@
       <c r="D9" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E9" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G9" s="4">
         <f>COUNTIF(B9:E9, TRUE)</f>
         <v>0</v>
@@ -2666,9 +2570,6 @@
       <c r="D10" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E10" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G10" s="4">
         <f>COUNTIF(B10:E10, TRUE)</f>
         <v>0</v>
@@ -2691,9 +2592,6 @@
       <c r="D11" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E11" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G11" s="4">
         <f>COUNTIF(B11:E11, TRUE)</f>
         <v>0</v>
@@ -2716,9 +2614,6 @@
       <c r="D12" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E12" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G12" s="4">
         <f>COUNTIF(B12:E12, TRUE)</f>
         <v>0</v>
@@ -2741,9 +2636,6 @@
       <c r="D13" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E13" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G13" s="4">
         <f>COUNTIF(B13:E13, TRUE)</f>
         <v>0</v>
@@ -2766,9 +2658,6 @@
       <c r="D14" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E14" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G14" s="4">
         <f>COUNTIF(B14:E14, TRUE)</f>
         <v>0</v>
@@ -2791,9 +2680,6 @@
       <c r="D15" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E15" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G15" s="4">
         <f>COUNTIF(B15:E15, TRUE)</f>
         <v>0</v>
@@ -2816,9 +2702,6 @@
       <c r="D16" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E16" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G16" s="4">
         <f>COUNTIF(B16:E16, TRUE)</f>
         <v>0</v>
@@ -2841,9 +2724,6 @@
       <c r="D17" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E17" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G17" s="4">
         <f>COUNTIF(B17:E17, TRUE)</f>
         <v>0</v>
@@ -2866,9 +2746,6 @@
       <c r="D18" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E18" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G18" s="4">
         <f>COUNTIF(B18:E18, TRUE)</f>
         <v>0</v>
@@ -2891,9 +2768,6 @@
       <c r="D19" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E19" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G19" s="4">
         <f>COUNTIF(B19:E19, TRUE)</f>
         <v>0</v>
@@ -2916,9 +2790,6 @@
       <c r="D20" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E20" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G20" s="4">
         <f>COUNTIF(B20:E20, TRUE)</f>
         <v>0</v>
@@ -2941,9 +2812,6 @@
       <c r="D21" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E21" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G21" s="4">
         <f>COUNTIF(B21:E21, TRUE)</f>
         <v>0</v>
@@ -2966,9 +2834,6 @@
       <c r="D22" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E22" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G22" s="4">
         <f>COUNTIF(B22:E22, TRUE)</f>
         <v>0</v>
@@ -2991,9 +2856,6 @@
       <c r="D23" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E23" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G23" s="4">
         <f>COUNTIF(B23:E23, TRUE)</f>
         <v>0</v>
@@ -3016,9 +2878,6 @@
       <c r="D24" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E24" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G24" s="4">
         <f>COUNTIF(B24:E24, TRUE)</f>
         <v>0</v>
@@ -3041,40 +2900,12 @@
       <c r="D25" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E25" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G25" s="4">
         <f>COUNTIF(B25:E25, TRUE)</f>
         <v>0</v>
       </c>
       <c r="H25" s="4">
         <f>COUNTIF(C25, TRUE)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8">
-      <c r="A26" t="s">
-        <v>41</v>
-      </c>
-      <c r="B26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="C26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="D26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="E26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="G26" s="4">
-        <f>COUNTIF(B26:E26, TRUE)</f>
-        <v>0</v>
-      </c>
-      <c r="H26" s="4">
-        <f>COUNTIF(C26, TRUE)</f>
         <v>0</v>
       </c>
     </row>
@@ -3085,7 +2916,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.140625" customWidth="1"/>
@@ -3098,25 +2929,25 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>48</v>
-      </c>
       <c r="G1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -3132,9 +2963,6 @@
       <c r="D2" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E2" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G2" s="4">
         <f>COUNTIF(B2:E2, TRUE)</f>
         <v>0</v>
@@ -3157,9 +2985,6 @@
       <c r="D3" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E3" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G3" s="4">
         <f>COUNTIF(B3:E3, TRUE)</f>
         <v>0</v>
@@ -3182,9 +3007,6 @@
       <c r="D4" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E4" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G4" s="4">
         <f>COUNTIF(B4:E4, TRUE)</f>
         <v>0</v>
@@ -3207,9 +3029,6 @@
       <c r="D5" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E5" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G5" s="4">
         <f>COUNTIF(B5:E5, TRUE)</f>
         <v>0</v>
@@ -3232,9 +3051,6 @@
       <c r="D6" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E6" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G6" s="4">
         <f>COUNTIF(B6:E6, TRUE)</f>
         <v>0</v>
@@ -3257,9 +3073,6 @@
       <c r="D7" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E7" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G7" s="4">
         <f>COUNTIF(B7:E7, TRUE)</f>
         <v>0</v>
@@ -3282,9 +3095,6 @@
       <c r="D8" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E8" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G8" s="4">
         <f>COUNTIF(B8:E8, TRUE)</f>
         <v>0</v>
@@ -3307,9 +3117,6 @@
       <c r="D9" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E9" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G9" s="4">
         <f>COUNTIF(B9:E9, TRUE)</f>
         <v>0</v>
@@ -3332,9 +3139,6 @@
       <c r="D10" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E10" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G10" s="4">
         <f>COUNTIF(B10:E10, TRUE)</f>
         <v>0</v>
@@ -3357,9 +3161,6 @@
       <c r="D11" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E11" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G11" s="4">
         <f>COUNTIF(B11:E11, TRUE)</f>
         <v>0</v>
@@ -3382,9 +3183,6 @@
       <c r="D12" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E12" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G12" s="4">
         <f>COUNTIF(B12:E12, TRUE)</f>
         <v>0</v>
@@ -3407,9 +3205,6 @@
       <c r="D13" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E13" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G13" s="4">
         <f>COUNTIF(B13:E13, TRUE)</f>
         <v>0</v>
@@ -3432,9 +3227,6 @@
       <c r="D14" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E14" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G14" s="4">
         <f>COUNTIF(B14:E14, TRUE)</f>
         <v>0</v>
@@ -3457,9 +3249,6 @@
       <c r="D15" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E15" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G15" s="4">
         <f>COUNTIF(B15:E15, TRUE)</f>
         <v>0</v>
@@ -3482,9 +3271,6 @@
       <c r="D16" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E16" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G16" s="4">
         <f>COUNTIF(B16:E16, TRUE)</f>
         <v>0</v>
@@ -3507,9 +3293,6 @@
       <c r="D17" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E17" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G17" s="4">
         <f>COUNTIF(B17:E17, TRUE)</f>
         <v>0</v>
@@ -3532,9 +3315,6 @@
       <c r="D18" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E18" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G18" s="4">
         <f>COUNTIF(B18:E18, TRUE)</f>
         <v>0</v>
@@ -3557,9 +3337,6 @@
       <c r="D19" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E19" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G19" s="4">
         <f>COUNTIF(B19:E19, TRUE)</f>
         <v>0</v>
@@ -3582,9 +3359,6 @@
       <c r="D20" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E20" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G20" s="4">
         <f>COUNTIF(B20:E20, TRUE)</f>
         <v>0</v>
@@ -3607,9 +3381,6 @@
       <c r="D21" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E21" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G21" s="4">
         <f>COUNTIF(B21:E21, TRUE)</f>
         <v>0</v>
@@ -3632,9 +3403,6 @@
       <c r="D22" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E22" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G22" s="4">
         <f>COUNTIF(B22:E22, TRUE)</f>
         <v>0</v>
@@ -3657,9 +3425,6 @@
       <c r="D23" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E23" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G23" s="4">
         <f>COUNTIF(B23:E23, TRUE)</f>
         <v>0</v>
@@ -3682,9 +3447,6 @@
       <c r="D24" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E24" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G24" s="4">
         <f>COUNTIF(B24:E24, TRUE)</f>
         <v>0</v>
@@ -3707,40 +3469,12 @@
       <c r="D25" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E25" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G25" s="4">
         <f>COUNTIF(B25:E25, TRUE)</f>
         <v>0</v>
       </c>
       <c r="H25" s="4">
         <f>COUNTIF(C25, TRUE)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8">
-      <c r="A26" t="s">
-        <v>41</v>
-      </c>
-      <c r="B26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="C26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="D26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="E26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="G26" s="4">
-        <f>COUNTIF(B26:E26, TRUE)</f>
-        <v>0</v>
-      </c>
-      <c r="H26" s="4">
-        <f>COUNTIF(C26, TRUE)</f>
         <v>0</v>
       </c>
     </row>
@@ -3751,7 +3485,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.140625" customWidth="1"/>
@@ -3764,25 +3498,25 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>48</v>
-      </c>
       <c r="G1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -3798,9 +3532,6 @@
       <c r="D2" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E2" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G2" s="4">
         <f>COUNTIF(B2:E2, TRUE)</f>
         <v>0</v>
@@ -3823,9 +3554,6 @@
       <c r="D3" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E3" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G3" s="4">
         <f>COUNTIF(B3:E3, TRUE)</f>
         <v>0</v>
@@ -3848,9 +3576,6 @@
       <c r="D4" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E4" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G4" s="4">
         <f>COUNTIF(B4:E4, TRUE)</f>
         <v>0</v>
@@ -3873,9 +3598,6 @@
       <c r="D5" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E5" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G5" s="4">
         <f>COUNTIF(B5:E5, TRUE)</f>
         <v>0</v>
@@ -3898,9 +3620,6 @@
       <c r="D6" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E6" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G6" s="4">
         <f>COUNTIF(B6:E6, TRUE)</f>
         <v>0</v>
@@ -3923,9 +3642,6 @@
       <c r="D7" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E7" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G7" s="4">
         <f>COUNTIF(B7:E7, TRUE)</f>
         <v>0</v>
@@ -3948,9 +3664,6 @@
       <c r="D8" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E8" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G8" s="4">
         <f>COUNTIF(B8:E8, TRUE)</f>
         <v>0</v>
@@ -3973,9 +3686,6 @@
       <c r="D9" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E9" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G9" s="4">
         <f>COUNTIF(B9:E9, TRUE)</f>
         <v>0</v>
@@ -3998,9 +3708,6 @@
       <c r="D10" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E10" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G10" s="4">
         <f>COUNTIF(B10:E10, TRUE)</f>
         <v>0</v>
@@ -4023,9 +3730,6 @@
       <c r="D11" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E11" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G11" s="4">
         <f>COUNTIF(B11:E11, TRUE)</f>
         <v>0</v>
@@ -4048,9 +3752,6 @@
       <c r="D12" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E12" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G12" s="4">
         <f>COUNTIF(B12:E12, TRUE)</f>
         <v>0</v>
@@ -4073,9 +3774,6 @@
       <c r="D13" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E13" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G13" s="4">
         <f>COUNTIF(B13:E13, TRUE)</f>
         <v>0</v>
@@ -4098,9 +3796,6 @@
       <c r="D14" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E14" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G14" s="4">
         <f>COUNTIF(B14:E14, TRUE)</f>
         <v>0</v>
@@ -4123,9 +3818,6 @@
       <c r="D15" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E15" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G15" s="4">
         <f>COUNTIF(B15:E15, TRUE)</f>
         <v>0</v>
@@ -4148,9 +3840,6 @@
       <c r="D16" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E16" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G16" s="4">
         <f>COUNTIF(B16:E16, TRUE)</f>
         <v>0</v>
@@ -4173,9 +3862,6 @@
       <c r="D17" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E17" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G17" s="4">
         <f>COUNTIF(B17:E17, TRUE)</f>
         <v>0</v>
@@ -4198,9 +3884,6 @@
       <c r="D18" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E18" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G18" s="4">
         <f>COUNTIF(B18:E18, TRUE)</f>
         <v>0</v>
@@ -4223,9 +3906,6 @@
       <c r="D19" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E19" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G19" s="4">
         <f>COUNTIF(B19:E19, TRUE)</f>
         <v>0</v>
@@ -4248,9 +3928,6 @@
       <c r="D20" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E20" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G20" s="4">
         <f>COUNTIF(B20:E20, TRUE)</f>
         <v>0</v>
@@ -4273,9 +3950,6 @@
       <c r="D21" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E21" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G21" s="4">
         <f>COUNTIF(B21:E21, TRUE)</f>
         <v>0</v>
@@ -4298,9 +3972,6 @@
       <c r="D22" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E22" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G22" s="4">
         <f>COUNTIF(B22:E22, TRUE)</f>
         <v>0</v>
@@ -4323,9 +3994,6 @@
       <c r="D23" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E23" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G23" s="4">
         <f>COUNTIF(B23:E23, TRUE)</f>
         <v>0</v>
@@ -4348,9 +4016,6 @@
       <c r="D24" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E24" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G24" s="4">
         <f>COUNTIF(B24:E24, TRUE)</f>
         <v>0</v>
@@ -4373,40 +4038,12 @@
       <c r="D25" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E25" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G25" s="4">
         <f>COUNTIF(B25:E25, TRUE)</f>
         <v>0</v>
       </c>
       <c r="H25" s="4">
         <f>COUNTIF(C25, TRUE)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8">
-      <c r="A26" t="s">
-        <v>41</v>
-      </c>
-      <c r="B26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="C26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="D26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="E26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="G26" s="4">
-        <f>COUNTIF(B26:E26, TRUE)</f>
-        <v>0</v>
-      </c>
-      <c r="H26" s="4">
-        <f>COUNTIF(C26, TRUE)</f>
         <v>0</v>
       </c>
     </row>
@@ -4417,7 +4054,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.140625" customWidth="1"/>
@@ -4430,25 +4067,25 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>48</v>
-      </c>
       <c r="G1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -4464,9 +4101,6 @@
       <c r="D2" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E2" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G2" s="4">
         <f>COUNTIF(B2:E2, TRUE)</f>
         <v>0</v>
@@ -4489,9 +4123,6 @@
       <c r="D3" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E3" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G3" s="4">
         <f>COUNTIF(B3:E3, TRUE)</f>
         <v>0</v>
@@ -4514,9 +4145,6 @@
       <c r="D4" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E4" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G4" s="4">
         <f>COUNTIF(B4:E4, TRUE)</f>
         <v>0</v>
@@ -4539,9 +4167,6 @@
       <c r="D5" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E5" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G5" s="4">
         <f>COUNTIF(B5:E5, TRUE)</f>
         <v>0</v>
@@ -4564,9 +4189,6 @@
       <c r="D6" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E6" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G6" s="4">
         <f>COUNTIF(B6:E6, TRUE)</f>
         <v>0</v>
@@ -4589,9 +4211,6 @@
       <c r="D7" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E7" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G7" s="4">
         <f>COUNTIF(B7:E7, TRUE)</f>
         <v>0</v>
@@ -4614,9 +4233,6 @@
       <c r="D8" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E8" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G8" s="4">
         <f>COUNTIF(B8:E8, TRUE)</f>
         <v>0</v>
@@ -4639,9 +4255,6 @@
       <c r="D9" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E9" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G9" s="4">
         <f>COUNTIF(B9:E9, TRUE)</f>
         <v>0</v>
@@ -4664,9 +4277,6 @@
       <c r="D10" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E10" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G10" s="4">
         <f>COUNTIF(B10:E10, TRUE)</f>
         <v>0</v>
@@ -4689,9 +4299,6 @@
       <c r="D11" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E11" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G11" s="4">
         <f>COUNTIF(B11:E11, TRUE)</f>
         <v>0</v>
@@ -4714,9 +4321,6 @@
       <c r="D12" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E12" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G12" s="4">
         <f>COUNTIF(B12:E12, TRUE)</f>
         <v>0</v>
@@ -4739,9 +4343,6 @@
       <c r="D13" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E13" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G13" s="4">
         <f>COUNTIF(B13:E13, TRUE)</f>
         <v>0</v>
@@ -4764,9 +4365,6 @@
       <c r="D14" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E14" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G14" s="4">
         <f>COUNTIF(B14:E14, TRUE)</f>
         <v>0</v>
@@ -4789,9 +4387,6 @@
       <c r="D15" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E15" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G15" s="4">
         <f>COUNTIF(B15:E15, TRUE)</f>
         <v>0</v>
@@ -4814,9 +4409,6 @@
       <c r="D16" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E16" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G16" s="4">
         <f>COUNTIF(B16:E16, TRUE)</f>
         <v>0</v>
@@ -4839,9 +4431,6 @@
       <c r="D17" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E17" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G17" s="4">
         <f>COUNTIF(B17:E17, TRUE)</f>
         <v>0</v>
@@ -4864,9 +4453,6 @@
       <c r="D18" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E18" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G18" s="4">
         <f>COUNTIF(B18:E18, TRUE)</f>
         <v>0</v>
@@ -4889,9 +4475,6 @@
       <c r="D19" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E19" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G19" s="4">
         <f>COUNTIF(B19:E19, TRUE)</f>
         <v>0</v>
@@ -4914,9 +4497,6 @@
       <c r="D20" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E20" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G20" s="4">
         <f>COUNTIF(B20:E20, TRUE)</f>
         <v>0</v>
@@ -4939,9 +4519,6 @@
       <c r="D21" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E21" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G21" s="4">
         <f>COUNTIF(B21:E21, TRUE)</f>
         <v>0</v>
@@ -4964,9 +4541,6 @@
       <c r="D22" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E22" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G22" s="4">
         <f>COUNTIF(B22:E22, TRUE)</f>
         <v>0</v>
@@ -4989,9 +4563,6 @@
       <c r="D23" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E23" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G23" s="4">
         <f>COUNTIF(B23:E23, TRUE)</f>
         <v>0</v>
@@ -5014,9 +4585,6 @@
       <c r="D24" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E24" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G24" s="4">
         <f>COUNTIF(B24:E24, TRUE)</f>
         <v>0</v>
@@ -5039,40 +4607,12 @@
       <c r="D25" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E25" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G25" s="4">
         <f>COUNTIF(B25:E25, TRUE)</f>
         <v>0</v>
       </c>
       <c r="H25" s="4">
         <f>COUNTIF(C25, TRUE)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8">
-      <c r="A26" t="s">
-        <v>41</v>
-      </c>
-      <c r="B26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="C26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="D26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="E26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="G26" s="4">
-        <f>COUNTIF(B26:E26, TRUE)</f>
-        <v>0</v>
-      </c>
-      <c r="H26" s="4">
-        <f>COUNTIF(C26, TRUE)</f>
         <v>0</v>
       </c>
     </row>
@@ -5083,7 +4623,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.140625" customWidth="1"/>
@@ -5096,25 +4636,25 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>48</v>
-      </c>
       <c r="G1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -5130,9 +4670,6 @@
       <c r="D2" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E2" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G2" s="4">
         <f>COUNTIF(B2:E2, TRUE)</f>
         <v>0</v>
@@ -5155,9 +4692,6 @@
       <c r="D3" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E3" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G3" s="4">
         <f>COUNTIF(B3:E3, TRUE)</f>
         <v>0</v>
@@ -5180,9 +4714,6 @@
       <c r="D4" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E4" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G4" s="4">
         <f>COUNTIF(B4:E4, TRUE)</f>
         <v>0</v>
@@ -5205,9 +4736,6 @@
       <c r="D5" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E5" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G5" s="4">
         <f>COUNTIF(B5:E5, TRUE)</f>
         <v>0</v>
@@ -5230,9 +4758,6 @@
       <c r="D6" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E6" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G6" s="4">
         <f>COUNTIF(B6:E6, TRUE)</f>
         <v>0</v>
@@ -5255,9 +4780,6 @@
       <c r="D7" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E7" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G7" s="4">
         <f>COUNTIF(B7:E7, TRUE)</f>
         <v>0</v>
@@ -5280,9 +4802,6 @@
       <c r="D8" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E8" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G8" s="4">
         <f>COUNTIF(B8:E8, TRUE)</f>
         <v>0</v>
@@ -5305,9 +4824,6 @@
       <c r="D9" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E9" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G9" s="4">
         <f>COUNTIF(B9:E9, TRUE)</f>
         <v>0</v>
@@ -5330,9 +4846,6 @@
       <c r="D10" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E10" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G10" s="4">
         <f>COUNTIF(B10:E10, TRUE)</f>
         <v>0</v>
@@ -5355,9 +4868,6 @@
       <c r="D11" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E11" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G11" s="4">
         <f>COUNTIF(B11:E11, TRUE)</f>
         <v>0</v>
@@ -5380,9 +4890,6 @@
       <c r="D12" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E12" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G12" s="4">
         <f>COUNTIF(B12:E12, TRUE)</f>
         <v>0</v>
@@ -5405,9 +4912,6 @@
       <c r="D13" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E13" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G13" s="4">
         <f>COUNTIF(B13:E13, TRUE)</f>
         <v>0</v>
@@ -5430,9 +4934,6 @@
       <c r="D14" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E14" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G14" s="4">
         <f>COUNTIF(B14:E14, TRUE)</f>
         <v>0</v>
@@ -5455,9 +4956,6 @@
       <c r="D15" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E15" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G15" s="4">
         <f>COUNTIF(B15:E15, TRUE)</f>
         <v>0</v>
@@ -5480,9 +4978,6 @@
       <c r="D16" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E16" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G16" s="4">
         <f>COUNTIF(B16:E16, TRUE)</f>
         <v>0</v>
@@ -5505,9 +5000,6 @@
       <c r="D17" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E17" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G17" s="4">
         <f>COUNTIF(B17:E17, TRUE)</f>
         <v>0</v>
@@ -5530,9 +5022,6 @@
       <c r="D18" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E18" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G18" s="4">
         <f>COUNTIF(B18:E18, TRUE)</f>
         <v>0</v>
@@ -5555,9 +5044,6 @@
       <c r="D19" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E19" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G19" s="4">
         <f>COUNTIF(B19:E19, TRUE)</f>
         <v>0</v>
@@ -5580,9 +5066,6 @@
       <c r="D20" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E20" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G20" s="4">
         <f>COUNTIF(B20:E20, TRUE)</f>
         <v>0</v>
@@ -5605,9 +5088,6 @@
       <c r="D21" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E21" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G21" s="4">
         <f>COUNTIF(B21:E21, TRUE)</f>
         <v>0</v>
@@ -5630,9 +5110,6 @@
       <c r="D22" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E22" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G22" s="4">
         <f>COUNTIF(B22:E22, TRUE)</f>
         <v>0</v>
@@ -5655,9 +5132,6 @@
       <c r="D23" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E23" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G23" s="4">
         <f>COUNTIF(B23:E23, TRUE)</f>
         <v>0</v>
@@ -5680,9 +5154,6 @@
       <c r="D24" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E24" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G24" s="4">
         <f>COUNTIF(B24:E24, TRUE)</f>
         <v>0</v>
@@ -5705,40 +5176,12 @@
       <c r="D25" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E25" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G25" s="4">
         <f>COUNTIF(B25:E25, TRUE)</f>
         <v>0</v>
       </c>
       <c r="H25" s="4">
         <f>COUNTIF(C25, TRUE)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8">
-      <c r="A26" t="s">
-        <v>41</v>
-      </c>
-      <c r="B26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="C26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="D26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="E26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="G26" s="4">
-        <f>COUNTIF(B26:E26, TRUE)</f>
-        <v>0</v>
-      </c>
-      <c r="H26" s="4">
-        <f>COUNTIF(C26, TRUE)</f>
         <v>0</v>
       </c>
     </row>
@@ -5749,7 +5192,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.140625" customWidth="1"/>
@@ -5762,25 +5205,25 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>48</v>
-      </c>
       <c r="G1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -5796,9 +5239,6 @@
       <c r="D2" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E2" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G2" s="4">
         <f>COUNTIF(B2:E2, TRUE)</f>
         <v>0</v>
@@ -5821,9 +5261,6 @@
       <c r="D3" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E3" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G3" s="4">
         <f>COUNTIF(B3:E3, TRUE)</f>
         <v>0</v>
@@ -5846,9 +5283,6 @@
       <c r="D4" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E4" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G4" s="4">
         <f>COUNTIF(B4:E4, TRUE)</f>
         <v>0</v>
@@ -5871,9 +5305,6 @@
       <c r="D5" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E5" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G5" s="4">
         <f>COUNTIF(B5:E5, TRUE)</f>
         <v>0</v>
@@ -5896,9 +5327,6 @@
       <c r="D6" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E6" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G6" s="4">
         <f>COUNTIF(B6:E6, TRUE)</f>
         <v>0</v>
@@ -5921,9 +5349,6 @@
       <c r="D7" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E7" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G7" s="4">
         <f>COUNTIF(B7:E7, TRUE)</f>
         <v>0</v>
@@ -5946,9 +5371,6 @@
       <c r="D8" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E8" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G8" s="4">
         <f>COUNTIF(B8:E8, TRUE)</f>
         <v>0</v>
@@ -5971,9 +5393,6 @@
       <c r="D9" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E9" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G9" s="4">
         <f>COUNTIF(B9:E9, TRUE)</f>
         <v>0</v>
@@ -5996,9 +5415,6 @@
       <c r="D10" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E10" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G10" s="4">
         <f>COUNTIF(B10:E10, TRUE)</f>
         <v>0</v>
@@ -6021,9 +5437,6 @@
       <c r="D11" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E11" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G11" s="4">
         <f>COUNTIF(B11:E11, TRUE)</f>
         <v>0</v>
@@ -6046,9 +5459,6 @@
       <c r="D12" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E12" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G12" s="4">
         <f>COUNTIF(B12:E12, TRUE)</f>
         <v>0</v>
@@ -6071,9 +5481,6 @@
       <c r="D13" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E13" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G13" s="4">
         <f>COUNTIF(B13:E13, TRUE)</f>
         <v>0</v>
@@ -6096,9 +5503,6 @@
       <c r="D14" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E14" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G14" s="4">
         <f>COUNTIF(B14:E14, TRUE)</f>
         <v>0</v>
@@ -6121,9 +5525,6 @@
       <c r="D15" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E15" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G15" s="4">
         <f>COUNTIF(B15:E15, TRUE)</f>
         <v>0</v>
@@ -6146,9 +5547,6 @@
       <c r="D16" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E16" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G16" s="4">
         <f>COUNTIF(B16:E16, TRUE)</f>
         <v>0</v>
@@ -6171,9 +5569,6 @@
       <c r="D17" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E17" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G17" s="4">
         <f>COUNTIF(B17:E17, TRUE)</f>
         <v>0</v>
@@ -6196,9 +5591,6 @@
       <c r="D18" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E18" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G18" s="4">
         <f>COUNTIF(B18:E18, TRUE)</f>
         <v>0</v>
@@ -6221,9 +5613,6 @@
       <c r="D19" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E19" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G19" s="4">
         <f>COUNTIF(B19:E19, TRUE)</f>
         <v>0</v>
@@ -6246,9 +5635,6 @@
       <c r="D20" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E20" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G20" s="4">
         <f>COUNTIF(B20:E20, TRUE)</f>
         <v>0</v>
@@ -6271,9 +5657,6 @@
       <c r="D21" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E21" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G21" s="4">
         <f>COUNTIF(B21:E21, TRUE)</f>
         <v>0</v>
@@ -6296,9 +5679,6 @@
       <c r="D22" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E22" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G22" s="4">
         <f>COUNTIF(B22:E22, TRUE)</f>
         <v>0</v>
@@ -6321,9 +5701,6 @@
       <c r="D23" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E23" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G23" s="4">
         <f>COUNTIF(B23:E23, TRUE)</f>
         <v>0</v>
@@ -6346,9 +5723,6 @@
       <c r="D24" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E24" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G24" s="4">
         <f>COUNTIF(B24:E24, TRUE)</f>
         <v>0</v>
@@ -6371,40 +5745,12 @@
       <c r="D25" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E25" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G25" s="4">
         <f>COUNTIF(B25:E25, TRUE)</f>
         <v>0</v>
       </c>
       <c r="H25" s="4">
         <f>COUNTIF(C25, TRUE)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8">
-      <c r="A26" t="s">
-        <v>41</v>
-      </c>
-      <c r="B26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="C26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="D26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="E26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="G26" s="4">
-        <f>COUNTIF(B26:E26, TRUE)</f>
-        <v>0</v>
-      </c>
-      <c r="H26" s="4">
-        <f>COUNTIF(C26, TRUE)</f>
         <v>0</v>
       </c>
     </row>
@@ -6415,7 +5761,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.140625" customWidth="1"/>
@@ -6428,25 +5774,25 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>48</v>
-      </c>
       <c r="G1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -6462,9 +5808,6 @@
       <c r="D2" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E2" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G2" s="4">
         <f>COUNTIF(B2:E2, TRUE)</f>
         <v>0</v>
@@ -6487,9 +5830,6 @@
       <c r="D3" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E3" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G3" s="4">
         <f>COUNTIF(B3:E3, TRUE)</f>
         <v>0</v>
@@ -6512,9 +5852,6 @@
       <c r="D4" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E4" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G4" s="4">
         <f>COUNTIF(B4:E4, TRUE)</f>
         <v>0</v>
@@ -6537,9 +5874,6 @@
       <c r="D5" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E5" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G5" s="4">
         <f>COUNTIF(B5:E5, TRUE)</f>
         <v>0</v>
@@ -6562,9 +5896,6 @@
       <c r="D6" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E6" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G6" s="4">
         <f>COUNTIF(B6:E6, TRUE)</f>
         <v>0</v>
@@ -6587,9 +5918,6 @@
       <c r="D7" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E7" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G7" s="4">
         <f>COUNTIF(B7:E7, TRUE)</f>
         <v>0</v>
@@ -6612,9 +5940,6 @@
       <c r="D8" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E8" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G8" s="4">
         <f>COUNTIF(B8:E8, TRUE)</f>
         <v>0</v>
@@ -6637,9 +5962,6 @@
       <c r="D9" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E9" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G9" s="4">
         <f>COUNTIF(B9:E9, TRUE)</f>
         <v>0</v>
@@ -6662,9 +5984,6 @@
       <c r="D10" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E10" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G10" s="4">
         <f>COUNTIF(B10:E10, TRUE)</f>
         <v>0</v>
@@ -6687,9 +6006,6 @@
       <c r="D11" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E11" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G11" s="4">
         <f>COUNTIF(B11:E11, TRUE)</f>
         <v>0</v>
@@ -6712,9 +6028,6 @@
       <c r="D12" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E12" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G12" s="4">
         <f>COUNTIF(B12:E12, TRUE)</f>
         <v>0</v>
@@ -6737,9 +6050,6 @@
       <c r="D13" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E13" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G13" s="4">
         <f>COUNTIF(B13:E13, TRUE)</f>
         <v>0</v>
@@ -6762,9 +6072,6 @@
       <c r="D14" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E14" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G14" s="4">
         <f>COUNTIF(B14:E14, TRUE)</f>
         <v>0</v>
@@ -6787,9 +6094,6 @@
       <c r="D15" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E15" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G15" s="4">
         <f>COUNTIF(B15:E15, TRUE)</f>
         <v>0</v>
@@ -6812,9 +6116,6 @@
       <c r="D16" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E16" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G16" s="4">
         <f>COUNTIF(B16:E16, TRUE)</f>
         <v>0</v>
@@ -6837,9 +6138,6 @@
       <c r="D17" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E17" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G17" s="4">
         <f>COUNTIF(B17:E17, TRUE)</f>
         <v>0</v>
@@ -6862,9 +6160,6 @@
       <c r="D18" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E18" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G18" s="4">
         <f>COUNTIF(B18:E18, TRUE)</f>
         <v>0</v>
@@ -6887,9 +6182,6 @@
       <c r="D19" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E19" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G19" s="4">
         <f>COUNTIF(B19:E19, TRUE)</f>
         <v>0</v>
@@ -6912,9 +6204,6 @@
       <c r="D20" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E20" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G20" s="4">
         <f>COUNTIF(B20:E20, TRUE)</f>
         <v>0</v>
@@ -6937,9 +6226,6 @@
       <c r="D21" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E21" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G21" s="4">
         <f>COUNTIF(B21:E21, TRUE)</f>
         <v>0</v>
@@ -6962,9 +6248,6 @@
       <c r="D22" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E22" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G22" s="4">
         <f>COUNTIF(B22:E22, TRUE)</f>
         <v>0</v>
@@ -6987,9 +6270,6 @@
       <c r="D23" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E23" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G23" s="4">
         <f>COUNTIF(B23:E23, TRUE)</f>
         <v>0</v>
@@ -7012,9 +6292,6 @@
       <c r="D24" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E24" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G24" s="4">
         <f>COUNTIF(B24:E24, TRUE)</f>
         <v>0</v>
@@ -7037,40 +6314,12 @@
       <c r="D25" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E25" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G25" s="4">
         <f>COUNTIF(B25:E25, TRUE)</f>
         <v>0</v>
       </c>
       <c r="H25" s="4">
         <f>COUNTIF(C25, TRUE)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8">
-      <c r="A26" t="s">
-        <v>41</v>
-      </c>
-      <c r="B26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="C26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="D26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="E26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="G26" s="4">
-        <f>COUNTIF(B26:E26, TRUE)</f>
-        <v>0</v>
-      </c>
-      <c r="H26" s="4">
-        <f>COUNTIF(C26, TRUE)</f>
         <v>0</v>
       </c>
     </row>
@@ -7081,7 +6330,7 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="26.7109375" customWidth="1"/>
@@ -7089,13 +6338,13 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -7407,19 +6656,6 @@
       </c>
       <c r="C25" s="5">
         <f>SUM('Week 1:Week 15'!H25) / 16</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3">
-      <c r="A26" t="s">
-        <v>41</v>
-      </c>
-      <c r="B26" s="4">
-        <f>SUM('Week 1:Week 15'!H26)</f>
-        <v>0</v>
-      </c>
-      <c r="C26" s="5">
-        <f>SUM('Week 1:Week 15'!H26) / 16</f>
         <v>0</v>
       </c>
     </row>
@@ -7430,7 +6666,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.140625" customWidth="1"/>
@@ -7443,25 +6679,25 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>48</v>
-      </c>
       <c r="G1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -7477,9 +6713,6 @@
       <c r="D2" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E2" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G2" s="4">
         <f>COUNTIF(B2:E2, TRUE)</f>
         <v>0</v>
@@ -7502,9 +6735,6 @@
       <c r="D3" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E3" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G3" s="4">
         <f>COUNTIF(B3:E3, TRUE)</f>
         <v>0</v>
@@ -7527,9 +6757,6 @@
       <c r="D4" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E4" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G4" s="4">
         <f>COUNTIF(B4:E4, TRUE)</f>
         <v>0</v>
@@ -7552,9 +6779,6 @@
       <c r="D5" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E5" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G5" s="4">
         <f>COUNTIF(B5:E5, TRUE)</f>
         <v>0</v>
@@ -7577,9 +6801,6 @@
       <c r="D6" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E6" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G6" s="4">
         <f>COUNTIF(B6:E6, TRUE)</f>
         <v>0</v>
@@ -7602,9 +6823,6 @@
       <c r="D7" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E7" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G7" s="4">
         <f>COUNTIF(B7:E7, TRUE)</f>
         <v>0</v>
@@ -7627,9 +6845,6 @@
       <c r="D8" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E8" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G8" s="4">
         <f>COUNTIF(B8:E8, TRUE)</f>
         <v>0</v>
@@ -7652,9 +6867,6 @@
       <c r="D9" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E9" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G9" s="4">
         <f>COUNTIF(B9:E9, TRUE)</f>
         <v>0</v>
@@ -7677,9 +6889,6 @@
       <c r="D10" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E10" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G10" s="4">
         <f>COUNTIF(B10:E10, TRUE)</f>
         <v>0</v>
@@ -7702,9 +6911,6 @@
       <c r="D11" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E11" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G11" s="4">
         <f>COUNTIF(B11:E11, TRUE)</f>
         <v>0</v>
@@ -7727,9 +6933,6 @@
       <c r="D12" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E12" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G12" s="4">
         <f>COUNTIF(B12:E12, TRUE)</f>
         <v>0</v>
@@ -7752,9 +6955,6 @@
       <c r="D13" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E13" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G13" s="4">
         <f>COUNTIF(B13:E13, TRUE)</f>
         <v>0</v>
@@ -7777,9 +6977,6 @@
       <c r="D14" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E14" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G14" s="4">
         <f>COUNTIF(B14:E14, TRUE)</f>
         <v>0</v>
@@ -7802,9 +6999,6 @@
       <c r="D15" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E15" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G15" s="4">
         <f>COUNTIF(B15:E15, TRUE)</f>
         <v>0</v>
@@ -7827,9 +7021,6 @@
       <c r="D16" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E16" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G16" s="4">
         <f>COUNTIF(B16:E16, TRUE)</f>
         <v>0</v>
@@ -7852,9 +7043,6 @@
       <c r="D17" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E17" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G17" s="4">
         <f>COUNTIF(B17:E17, TRUE)</f>
         <v>0</v>
@@ -7877,9 +7065,6 @@
       <c r="D18" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E18" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G18" s="4">
         <f>COUNTIF(B18:E18, TRUE)</f>
         <v>0</v>
@@ -7902,9 +7087,6 @@
       <c r="D19" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E19" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G19" s="4">
         <f>COUNTIF(B19:E19, TRUE)</f>
         <v>0</v>
@@ -7927,9 +7109,6 @@
       <c r="D20" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E20" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G20" s="4">
         <f>COUNTIF(B20:E20, TRUE)</f>
         <v>0</v>
@@ -7952,9 +7131,6 @@
       <c r="D21" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E21" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G21" s="4">
         <f>COUNTIF(B21:E21, TRUE)</f>
         <v>0</v>
@@ -7977,9 +7153,6 @@
       <c r="D22" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E22" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G22" s="4">
         <f>COUNTIF(B22:E22, TRUE)</f>
         <v>0</v>
@@ -8002,9 +7175,6 @@
       <c r="D23" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E23" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G23" s="4">
         <f>COUNTIF(B23:E23, TRUE)</f>
         <v>0</v>
@@ -8027,9 +7197,6 @@
       <c r="D24" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E24" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G24" s="4">
         <f>COUNTIF(B24:E24, TRUE)</f>
         <v>0</v>
@@ -8052,40 +7219,12 @@
       <c r="D25" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E25" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G25" s="4">
         <f>COUNTIF(B25:E25, TRUE)</f>
         <v>0</v>
       </c>
       <c r="H25" s="4">
         <f>COUNTIF(C25, TRUE)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8">
-      <c r="A26" t="s">
-        <v>41</v>
-      </c>
-      <c r="B26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="C26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="D26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="E26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="G26" s="4">
-        <f>COUNTIF(B26:E26, TRUE)</f>
-        <v>0</v>
-      </c>
-      <c r="H26" s="4">
-        <f>COUNTIF(C26, TRUE)</f>
         <v>0</v>
       </c>
     </row>
@@ -8096,7 +7235,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.140625" customWidth="1"/>
@@ -8109,25 +7248,25 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>48</v>
-      </c>
       <c r="G1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -8143,9 +7282,6 @@
       <c r="D2" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E2" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G2" s="4">
         <f>COUNTIF(B2:E2, TRUE)</f>
         <v>0</v>
@@ -8168,9 +7304,6 @@
       <c r="D3" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E3" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G3" s="4">
         <f>COUNTIF(B3:E3, TRUE)</f>
         <v>0</v>
@@ -8193,9 +7326,6 @@
       <c r="D4" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E4" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G4" s="4">
         <f>COUNTIF(B4:E4, TRUE)</f>
         <v>0</v>
@@ -8218,9 +7348,6 @@
       <c r="D5" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E5" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G5" s="4">
         <f>COUNTIF(B5:E5, TRUE)</f>
         <v>0</v>
@@ -8243,9 +7370,6 @@
       <c r="D6" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E6" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G6" s="4">
         <f>COUNTIF(B6:E6, TRUE)</f>
         <v>0</v>
@@ -8268,9 +7392,6 @@
       <c r="D7" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E7" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G7" s="4">
         <f>COUNTIF(B7:E7, TRUE)</f>
         <v>0</v>
@@ -8293,9 +7414,6 @@
       <c r="D8" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E8" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G8" s="4">
         <f>COUNTIF(B8:E8, TRUE)</f>
         <v>0</v>
@@ -8318,9 +7436,6 @@
       <c r="D9" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E9" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G9" s="4">
         <f>COUNTIF(B9:E9, TRUE)</f>
         <v>0</v>
@@ -8343,9 +7458,6 @@
       <c r="D10" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E10" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G10" s="4">
         <f>COUNTIF(B10:E10, TRUE)</f>
         <v>0</v>
@@ -8368,9 +7480,6 @@
       <c r="D11" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E11" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G11" s="4">
         <f>COUNTIF(B11:E11, TRUE)</f>
         <v>0</v>
@@ -8393,9 +7502,6 @@
       <c r="D12" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E12" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G12" s="4">
         <f>COUNTIF(B12:E12, TRUE)</f>
         <v>0</v>
@@ -8418,9 +7524,6 @@
       <c r="D13" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E13" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G13" s="4">
         <f>COUNTIF(B13:E13, TRUE)</f>
         <v>0</v>
@@ -8443,9 +7546,6 @@
       <c r="D14" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E14" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G14" s="4">
         <f>COUNTIF(B14:E14, TRUE)</f>
         <v>0</v>
@@ -8468,9 +7568,6 @@
       <c r="D15" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E15" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G15" s="4">
         <f>COUNTIF(B15:E15, TRUE)</f>
         <v>0</v>
@@ -8493,9 +7590,6 @@
       <c r="D16" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E16" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G16" s="4">
         <f>COUNTIF(B16:E16, TRUE)</f>
         <v>0</v>
@@ -8518,9 +7612,6 @@
       <c r="D17" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E17" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G17" s="4">
         <f>COUNTIF(B17:E17, TRUE)</f>
         <v>0</v>
@@ -8543,9 +7634,6 @@
       <c r="D18" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E18" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G18" s="4">
         <f>COUNTIF(B18:E18, TRUE)</f>
         <v>0</v>
@@ -8568,9 +7656,6 @@
       <c r="D19" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E19" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G19" s="4">
         <f>COUNTIF(B19:E19, TRUE)</f>
         <v>0</v>
@@ -8593,9 +7678,6 @@
       <c r="D20" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E20" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G20" s="4">
         <f>COUNTIF(B20:E20, TRUE)</f>
         <v>0</v>
@@ -8618,9 +7700,6 @@
       <c r="D21" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E21" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G21" s="4">
         <f>COUNTIF(B21:E21, TRUE)</f>
         <v>0</v>
@@ -8643,9 +7722,6 @@
       <c r="D22" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E22" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G22" s="4">
         <f>COUNTIF(B22:E22, TRUE)</f>
         <v>0</v>
@@ -8668,9 +7744,6 @@
       <c r="D23" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E23" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G23" s="4">
         <f>COUNTIF(B23:E23, TRUE)</f>
         <v>0</v>
@@ -8693,9 +7766,6 @@
       <c r="D24" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E24" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G24" s="4">
         <f>COUNTIF(B24:E24, TRUE)</f>
         <v>0</v>
@@ -8718,40 +7788,12 @@
       <c r="D25" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E25" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G25" s="4">
         <f>COUNTIF(B25:E25, TRUE)</f>
         <v>0</v>
       </c>
       <c r="H25" s="4">
         <f>COUNTIF(C25, TRUE)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8">
-      <c r="A26" t="s">
-        <v>41</v>
-      </c>
-      <c r="B26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="C26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="D26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="E26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="G26" s="4">
-        <f>COUNTIF(B26:E26, TRUE)</f>
-        <v>0</v>
-      </c>
-      <c r="H26" s="4">
-        <f>COUNTIF(C26, TRUE)</f>
         <v>0</v>
       </c>
     </row>
@@ -8762,7 +7804,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.140625" customWidth="1"/>
@@ -8775,25 +7817,25 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>48</v>
-      </c>
       <c r="G1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -8809,9 +7851,6 @@
       <c r="D2" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E2" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G2" s="4">
         <f>COUNTIF(B2:E2, TRUE)</f>
         <v>0</v>
@@ -8834,9 +7873,6 @@
       <c r="D3" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E3" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G3" s="4">
         <f>COUNTIF(B3:E3, TRUE)</f>
         <v>0</v>
@@ -8859,9 +7895,6 @@
       <c r="D4" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E4" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G4" s="4">
         <f>COUNTIF(B4:E4, TRUE)</f>
         <v>0</v>
@@ -8884,9 +7917,6 @@
       <c r="D5" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E5" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G5" s="4">
         <f>COUNTIF(B5:E5, TRUE)</f>
         <v>0</v>
@@ -8909,9 +7939,6 @@
       <c r="D6" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E6" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G6" s="4">
         <f>COUNTIF(B6:E6, TRUE)</f>
         <v>0</v>
@@ -8934,9 +7961,6 @@
       <c r="D7" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E7" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G7" s="4">
         <f>COUNTIF(B7:E7, TRUE)</f>
         <v>0</v>
@@ -8959,9 +7983,6 @@
       <c r="D8" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E8" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G8" s="4">
         <f>COUNTIF(B8:E8, TRUE)</f>
         <v>0</v>
@@ -8984,9 +8005,6 @@
       <c r="D9" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E9" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G9" s="4">
         <f>COUNTIF(B9:E9, TRUE)</f>
         <v>0</v>
@@ -9009,9 +8027,6 @@
       <c r="D10" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E10" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G10" s="4">
         <f>COUNTIF(B10:E10, TRUE)</f>
         <v>0</v>
@@ -9034,9 +8049,6 @@
       <c r="D11" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E11" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G11" s="4">
         <f>COUNTIF(B11:E11, TRUE)</f>
         <v>0</v>
@@ -9059,9 +8071,6 @@
       <c r="D12" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E12" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G12" s="4">
         <f>COUNTIF(B12:E12, TRUE)</f>
         <v>0</v>
@@ -9084,9 +8093,6 @@
       <c r="D13" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E13" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G13" s="4">
         <f>COUNTIF(B13:E13, TRUE)</f>
         <v>0</v>
@@ -9109,9 +8115,6 @@
       <c r="D14" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E14" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G14" s="4">
         <f>COUNTIF(B14:E14, TRUE)</f>
         <v>0</v>
@@ -9134,9 +8137,6 @@
       <c r="D15" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E15" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G15" s="4">
         <f>COUNTIF(B15:E15, TRUE)</f>
         <v>0</v>
@@ -9159,9 +8159,6 @@
       <c r="D16" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E16" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G16" s="4">
         <f>COUNTIF(B16:E16, TRUE)</f>
         <v>0</v>
@@ -9184,9 +8181,6 @@
       <c r="D17" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E17" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G17" s="4">
         <f>COUNTIF(B17:E17, TRUE)</f>
         <v>0</v>
@@ -9209,9 +8203,6 @@
       <c r="D18" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E18" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G18" s="4">
         <f>COUNTIF(B18:E18, TRUE)</f>
         <v>0</v>
@@ -9234,9 +8225,6 @@
       <c r="D19" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E19" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G19" s="4">
         <f>COUNTIF(B19:E19, TRUE)</f>
         <v>0</v>
@@ -9259,9 +8247,6 @@
       <c r="D20" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E20" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G20" s="4">
         <f>COUNTIF(B20:E20, TRUE)</f>
         <v>0</v>
@@ -9284,9 +8269,6 @@
       <c r="D21" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E21" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G21" s="4">
         <f>COUNTIF(B21:E21, TRUE)</f>
         <v>0</v>
@@ -9309,9 +8291,6 @@
       <c r="D22" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E22" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G22" s="4">
         <f>COUNTIF(B22:E22, TRUE)</f>
         <v>0</v>
@@ -9334,9 +8313,6 @@
       <c r="D23" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E23" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G23" s="4">
         <f>COUNTIF(B23:E23, TRUE)</f>
         <v>0</v>
@@ -9359,9 +8335,6 @@
       <c r="D24" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E24" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G24" s="4">
         <f>COUNTIF(B24:E24, TRUE)</f>
         <v>0</v>
@@ -9384,40 +8357,12 @@
       <c r="D25" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E25" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G25" s="4">
         <f>COUNTIF(B25:E25, TRUE)</f>
         <v>0</v>
       </c>
       <c r="H25" s="4">
         <f>COUNTIF(C25, TRUE)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8">
-      <c r="A26" t="s">
-        <v>41</v>
-      </c>
-      <c r="B26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="C26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="D26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="E26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="G26" s="4">
-        <f>COUNTIF(B26:E26, TRUE)</f>
-        <v>0</v>
-      </c>
-      <c r="H26" s="4">
-        <f>COUNTIF(C26, TRUE)</f>
         <v>0</v>
       </c>
     </row>
@@ -9428,7 +8373,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.140625" customWidth="1"/>
@@ -9441,25 +8386,25 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>48</v>
-      </c>
       <c r="G1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -9475,9 +8420,6 @@
       <c r="D2" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E2" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G2" s="4">
         <f>COUNTIF(B2:E2, TRUE)</f>
         <v>0</v>
@@ -9500,9 +8442,6 @@
       <c r="D3" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E3" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G3" s="4">
         <f>COUNTIF(B3:E3, TRUE)</f>
         <v>0</v>
@@ -9525,9 +8464,6 @@
       <c r="D4" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E4" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G4" s="4">
         <f>COUNTIF(B4:E4, TRUE)</f>
         <v>0</v>
@@ -9550,9 +8486,6 @@
       <c r="D5" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E5" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G5" s="4">
         <f>COUNTIF(B5:E5, TRUE)</f>
         <v>0</v>
@@ -9575,9 +8508,6 @@
       <c r="D6" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E6" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G6" s="4">
         <f>COUNTIF(B6:E6, TRUE)</f>
         <v>0</v>
@@ -9600,9 +8530,6 @@
       <c r="D7" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E7" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G7" s="4">
         <f>COUNTIF(B7:E7, TRUE)</f>
         <v>0</v>
@@ -9625,9 +8552,6 @@
       <c r="D8" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E8" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G8" s="4">
         <f>COUNTIF(B8:E8, TRUE)</f>
         <v>0</v>
@@ -9650,9 +8574,6 @@
       <c r="D9" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E9" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G9" s="4">
         <f>COUNTIF(B9:E9, TRUE)</f>
         <v>0</v>
@@ -9675,9 +8596,6 @@
       <c r="D10" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E10" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G10" s="4">
         <f>COUNTIF(B10:E10, TRUE)</f>
         <v>0</v>
@@ -9700,9 +8618,6 @@
       <c r="D11" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E11" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G11" s="4">
         <f>COUNTIF(B11:E11, TRUE)</f>
         <v>0</v>
@@ -9725,9 +8640,6 @@
       <c r="D12" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E12" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G12" s="4">
         <f>COUNTIF(B12:E12, TRUE)</f>
         <v>0</v>
@@ -9750,9 +8662,6 @@
       <c r="D13" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E13" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G13" s="4">
         <f>COUNTIF(B13:E13, TRUE)</f>
         <v>0</v>
@@ -9775,9 +8684,6 @@
       <c r="D14" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E14" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G14" s="4">
         <f>COUNTIF(B14:E14, TRUE)</f>
         <v>0</v>
@@ -9800,9 +8706,6 @@
       <c r="D15" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E15" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G15" s="4">
         <f>COUNTIF(B15:E15, TRUE)</f>
         <v>0</v>
@@ -9825,9 +8728,6 @@
       <c r="D16" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E16" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G16" s="4">
         <f>COUNTIF(B16:E16, TRUE)</f>
         <v>0</v>
@@ -9850,9 +8750,6 @@
       <c r="D17" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E17" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G17" s="4">
         <f>COUNTIF(B17:E17, TRUE)</f>
         <v>0</v>
@@ -9875,9 +8772,6 @@
       <c r="D18" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E18" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G18" s="4">
         <f>COUNTIF(B18:E18, TRUE)</f>
         <v>0</v>
@@ -9900,9 +8794,6 @@
       <c r="D19" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E19" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G19" s="4">
         <f>COUNTIF(B19:E19, TRUE)</f>
         <v>0</v>
@@ -9925,9 +8816,6 @@
       <c r="D20" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E20" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G20" s="4">
         <f>COUNTIF(B20:E20, TRUE)</f>
         <v>0</v>
@@ -9950,9 +8838,6 @@
       <c r="D21" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E21" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G21" s="4">
         <f>COUNTIF(B21:E21, TRUE)</f>
         <v>0</v>
@@ -9975,9 +8860,6 @@
       <c r="D22" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E22" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G22" s="4">
         <f>COUNTIF(B22:E22, TRUE)</f>
         <v>0</v>
@@ -10000,9 +8882,6 @@
       <c r="D23" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E23" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G23" s="4">
         <f>COUNTIF(B23:E23, TRUE)</f>
         <v>0</v>
@@ -10025,9 +8904,6 @@
       <c r="D24" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E24" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G24" s="4">
         <f>COUNTIF(B24:E24, TRUE)</f>
         <v>0</v>
@@ -10050,40 +8926,12 @@
       <c r="D25" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E25" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G25" s="4">
         <f>COUNTIF(B25:E25, TRUE)</f>
         <v>0</v>
       </c>
       <c r="H25" s="4">
         <f>COUNTIF(C25, TRUE)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8">
-      <c r="A26" t="s">
-        <v>41</v>
-      </c>
-      <c r="B26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="C26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="D26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="E26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="G26" s="4">
-        <f>COUNTIF(B26:E26, TRUE)</f>
-        <v>0</v>
-      </c>
-      <c r="H26" s="4">
-        <f>COUNTIF(C26, TRUE)</f>
         <v>0</v>
       </c>
     </row>
@@ -10094,7 +8942,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.140625" customWidth="1"/>
@@ -10107,25 +8955,25 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>48</v>
-      </c>
       <c r="G1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -10141,9 +8989,6 @@
       <c r="D2" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E2" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G2" s="4">
         <f>COUNTIF(B2:E2, TRUE)</f>
         <v>0</v>
@@ -10166,9 +9011,6 @@
       <c r="D3" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E3" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G3" s="4">
         <f>COUNTIF(B3:E3, TRUE)</f>
         <v>0</v>
@@ -10191,9 +9033,6 @@
       <c r="D4" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E4" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G4" s="4">
         <f>COUNTIF(B4:E4, TRUE)</f>
         <v>0</v>
@@ -10216,9 +9055,6 @@
       <c r="D5" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E5" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G5" s="4">
         <f>COUNTIF(B5:E5, TRUE)</f>
         <v>0</v>
@@ -10241,9 +9077,6 @@
       <c r="D6" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E6" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G6" s="4">
         <f>COUNTIF(B6:E6, TRUE)</f>
         <v>0</v>
@@ -10266,9 +9099,6 @@
       <c r="D7" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E7" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G7" s="4">
         <f>COUNTIF(B7:E7, TRUE)</f>
         <v>0</v>
@@ -10291,9 +9121,6 @@
       <c r="D8" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E8" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G8" s="4">
         <f>COUNTIF(B8:E8, TRUE)</f>
         <v>0</v>
@@ -10316,9 +9143,6 @@
       <c r="D9" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E9" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G9" s="4">
         <f>COUNTIF(B9:E9, TRUE)</f>
         <v>0</v>
@@ -10341,9 +9165,6 @@
       <c r="D10" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E10" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G10" s="4">
         <f>COUNTIF(B10:E10, TRUE)</f>
         <v>0</v>
@@ -10366,9 +9187,6 @@
       <c r="D11" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E11" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G11" s="4">
         <f>COUNTIF(B11:E11, TRUE)</f>
         <v>0</v>
@@ -10391,9 +9209,6 @@
       <c r="D12" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E12" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G12" s="4">
         <f>COUNTIF(B12:E12, TRUE)</f>
         <v>0</v>
@@ -10416,9 +9231,6 @@
       <c r="D13" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E13" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G13" s="4">
         <f>COUNTIF(B13:E13, TRUE)</f>
         <v>0</v>
@@ -10441,9 +9253,6 @@
       <c r="D14" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E14" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G14" s="4">
         <f>COUNTIF(B14:E14, TRUE)</f>
         <v>0</v>
@@ -10466,9 +9275,6 @@
       <c r="D15" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E15" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G15" s="4">
         <f>COUNTIF(B15:E15, TRUE)</f>
         <v>0</v>
@@ -10491,9 +9297,6 @@
       <c r="D16" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E16" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G16" s="4">
         <f>COUNTIF(B16:E16, TRUE)</f>
         <v>0</v>
@@ -10516,9 +9319,6 @@
       <c r="D17" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E17" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G17" s="4">
         <f>COUNTIF(B17:E17, TRUE)</f>
         <v>0</v>
@@ -10541,9 +9341,6 @@
       <c r="D18" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E18" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G18" s="4">
         <f>COUNTIF(B18:E18, TRUE)</f>
         <v>0</v>
@@ -10566,9 +9363,6 @@
       <c r="D19" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E19" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G19" s="4">
         <f>COUNTIF(B19:E19, TRUE)</f>
         <v>0</v>
@@ -10591,9 +9385,6 @@
       <c r="D20" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E20" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G20" s="4">
         <f>COUNTIF(B20:E20, TRUE)</f>
         <v>0</v>
@@ -10616,9 +9407,6 @@
       <c r="D21" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E21" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G21" s="4">
         <f>COUNTIF(B21:E21, TRUE)</f>
         <v>0</v>
@@ -10641,9 +9429,6 @@
       <c r="D22" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E22" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G22" s="4">
         <f>COUNTIF(B22:E22, TRUE)</f>
         <v>0</v>
@@ -10666,9 +9451,6 @@
       <c r="D23" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E23" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G23" s="4">
         <f>COUNTIF(B23:E23, TRUE)</f>
         <v>0</v>
@@ -10691,9 +9473,6 @@
       <c r="D24" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E24" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G24" s="4">
         <f>COUNTIF(B24:E24, TRUE)</f>
         <v>0</v>
@@ -10716,40 +9495,12 @@
       <c r="D25" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E25" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G25" s="4">
         <f>COUNTIF(B25:E25, TRUE)</f>
         <v>0</v>
       </c>
       <c r="H25" s="4">
         <f>COUNTIF(C25, TRUE)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8">
-      <c r="A26" t="s">
-        <v>41</v>
-      </c>
-      <c r="B26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="C26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="D26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="E26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="G26" s="4">
-        <f>COUNTIF(B26:E26, TRUE)</f>
-        <v>0</v>
-      </c>
-      <c r="H26" s="4">
-        <f>COUNTIF(C26, TRUE)</f>
         <v>0</v>
       </c>
     </row>
@@ -10760,7 +9511,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.140625" customWidth="1"/>
@@ -10773,25 +9524,25 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>48</v>
-      </c>
       <c r="G1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -10807,9 +9558,6 @@
       <c r="D2" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E2" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G2" s="4">
         <f>COUNTIF(B2:E2, TRUE)</f>
         <v>0</v>
@@ -10832,9 +9580,6 @@
       <c r="D3" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E3" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G3" s="4">
         <f>COUNTIF(B3:E3, TRUE)</f>
         <v>0</v>
@@ -10857,9 +9602,6 @@
       <c r="D4" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E4" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G4" s="4">
         <f>COUNTIF(B4:E4, TRUE)</f>
         <v>0</v>
@@ -10882,9 +9624,6 @@
       <c r="D5" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E5" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G5" s="4">
         <f>COUNTIF(B5:E5, TRUE)</f>
         <v>0</v>
@@ -10907,9 +9646,6 @@
       <c r="D6" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E6" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G6" s="4">
         <f>COUNTIF(B6:E6, TRUE)</f>
         <v>0</v>
@@ -10932,9 +9668,6 @@
       <c r="D7" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E7" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G7" s="4">
         <f>COUNTIF(B7:E7, TRUE)</f>
         <v>0</v>
@@ -10957,9 +9690,6 @@
       <c r="D8" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E8" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G8" s="4">
         <f>COUNTIF(B8:E8, TRUE)</f>
         <v>0</v>
@@ -10982,9 +9712,6 @@
       <c r="D9" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E9" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G9" s="4">
         <f>COUNTIF(B9:E9, TRUE)</f>
         <v>0</v>
@@ -11007,9 +9734,6 @@
       <c r="D10" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E10" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G10" s="4">
         <f>COUNTIF(B10:E10, TRUE)</f>
         <v>0</v>
@@ -11032,9 +9756,6 @@
       <c r="D11" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E11" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G11" s="4">
         <f>COUNTIF(B11:E11, TRUE)</f>
         <v>0</v>
@@ -11057,9 +9778,6 @@
       <c r="D12" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E12" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G12" s="4">
         <f>COUNTIF(B12:E12, TRUE)</f>
         <v>0</v>
@@ -11082,9 +9800,6 @@
       <c r="D13" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E13" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G13" s="4">
         <f>COUNTIF(B13:E13, TRUE)</f>
         <v>0</v>
@@ -11107,9 +9822,6 @@
       <c r="D14" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E14" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G14" s="4">
         <f>COUNTIF(B14:E14, TRUE)</f>
         <v>0</v>
@@ -11132,9 +9844,6 @@
       <c r="D15" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E15" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G15" s="4">
         <f>COUNTIF(B15:E15, TRUE)</f>
         <v>0</v>
@@ -11157,9 +9866,6 @@
       <c r="D16" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E16" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G16" s="4">
         <f>COUNTIF(B16:E16, TRUE)</f>
         <v>0</v>
@@ -11182,9 +9888,6 @@
       <c r="D17" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E17" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G17" s="4">
         <f>COUNTIF(B17:E17, TRUE)</f>
         <v>0</v>
@@ -11207,9 +9910,6 @@
       <c r="D18" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E18" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G18" s="4">
         <f>COUNTIF(B18:E18, TRUE)</f>
         <v>0</v>
@@ -11232,9 +9932,6 @@
       <c r="D19" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E19" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G19" s="4">
         <f>COUNTIF(B19:E19, TRUE)</f>
         <v>0</v>
@@ -11257,9 +9954,6 @@
       <c r="D20" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E20" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G20" s="4">
         <f>COUNTIF(B20:E20, TRUE)</f>
         <v>0</v>
@@ -11282,9 +9976,6 @@
       <c r="D21" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E21" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G21" s="4">
         <f>COUNTIF(B21:E21, TRUE)</f>
         <v>0</v>
@@ -11307,9 +9998,6 @@
       <c r="D22" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E22" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G22" s="4">
         <f>COUNTIF(B22:E22, TRUE)</f>
         <v>0</v>
@@ -11332,9 +10020,6 @@
       <c r="D23" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E23" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G23" s="4">
         <f>COUNTIF(B23:E23, TRUE)</f>
         <v>0</v>
@@ -11357,9 +10042,6 @@
       <c r="D24" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E24" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G24" s="4">
         <f>COUNTIF(B24:E24, TRUE)</f>
         <v>0</v>
@@ -11382,40 +10064,12 @@
       <c r="D25" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E25" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G25" s="4">
         <f>COUNTIF(B25:E25, TRUE)</f>
         <v>0</v>
       </c>
       <c r="H25" s="4">
         <f>COUNTIF(C25, TRUE)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8">
-      <c r="A26" t="s">
-        <v>41</v>
-      </c>
-      <c r="B26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="C26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="D26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="E26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="G26" s="4">
-        <f>COUNTIF(B26:E26, TRUE)</f>
-        <v>0</v>
-      </c>
-      <c r="H26" s="4">
-        <f>COUNTIF(C26, TRUE)</f>
         <v>0</v>
       </c>
     </row>
@@ -11426,7 +10080,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.140625" customWidth="1"/>
@@ -11439,25 +10093,25 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>48</v>
-      </c>
       <c r="G1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -11473,9 +10127,6 @@
       <c r="D2" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E2" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G2" s="4">
         <f>COUNTIF(B2:E2, TRUE)</f>
         <v>0</v>
@@ -11498,9 +10149,6 @@
       <c r="D3" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E3" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G3" s="4">
         <f>COUNTIF(B3:E3, TRUE)</f>
         <v>0</v>
@@ -11523,9 +10171,6 @@
       <c r="D4" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E4" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G4" s="4">
         <f>COUNTIF(B4:E4, TRUE)</f>
         <v>0</v>
@@ -11548,9 +10193,6 @@
       <c r="D5" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E5" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G5" s="4">
         <f>COUNTIF(B5:E5, TRUE)</f>
         <v>0</v>
@@ -11573,9 +10215,6 @@
       <c r="D6" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E6" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G6" s="4">
         <f>COUNTIF(B6:E6, TRUE)</f>
         <v>0</v>
@@ -11598,9 +10237,6 @@
       <c r="D7" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E7" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G7" s="4">
         <f>COUNTIF(B7:E7, TRUE)</f>
         <v>0</v>
@@ -11623,9 +10259,6 @@
       <c r="D8" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E8" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G8" s="4">
         <f>COUNTIF(B8:E8, TRUE)</f>
         <v>0</v>
@@ -11648,9 +10281,6 @@
       <c r="D9" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E9" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G9" s="4">
         <f>COUNTIF(B9:E9, TRUE)</f>
         <v>0</v>
@@ -11673,9 +10303,6 @@
       <c r="D10" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E10" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G10" s="4">
         <f>COUNTIF(B10:E10, TRUE)</f>
         <v>0</v>
@@ -11698,9 +10325,6 @@
       <c r="D11" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E11" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G11" s="4">
         <f>COUNTIF(B11:E11, TRUE)</f>
         <v>0</v>
@@ -11723,9 +10347,6 @@
       <c r="D12" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E12" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G12" s="4">
         <f>COUNTIF(B12:E12, TRUE)</f>
         <v>0</v>
@@ -11748,9 +10369,6 @@
       <c r="D13" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E13" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G13" s="4">
         <f>COUNTIF(B13:E13, TRUE)</f>
         <v>0</v>
@@ -11773,9 +10391,6 @@
       <c r="D14" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E14" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G14" s="4">
         <f>COUNTIF(B14:E14, TRUE)</f>
         <v>0</v>
@@ -11798,9 +10413,6 @@
       <c r="D15" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E15" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G15" s="4">
         <f>COUNTIF(B15:E15, TRUE)</f>
         <v>0</v>
@@ -11823,9 +10435,6 @@
       <c r="D16" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E16" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G16" s="4">
         <f>COUNTIF(B16:E16, TRUE)</f>
         <v>0</v>
@@ -11848,9 +10457,6 @@
       <c r="D17" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E17" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G17" s="4">
         <f>COUNTIF(B17:E17, TRUE)</f>
         <v>0</v>
@@ -11873,9 +10479,6 @@
       <c r="D18" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E18" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G18" s="4">
         <f>COUNTIF(B18:E18, TRUE)</f>
         <v>0</v>
@@ -11898,9 +10501,6 @@
       <c r="D19" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E19" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G19" s="4">
         <f>COUNTIF(B19:E19, TRUE)</f>
         <v>0</v>
@@ -11923,9 +10523,6 @@
       <c r="D20" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E20" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G20" s="4">
         <f>COUNTIF(B20:E20, TRUE)</f>
         <v>0</v>
@@ -11948,9 +10545,6 @@
       <c r="D21" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E21" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G21" s="4">
         <f>COUNTIF(B21:E21, TRUE)</f>
         <v>0</v>
@@ -11973,9 +10567,6 @@
       <c r="D22" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E22" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G22" s="4">
         <f>COUNTIF(B22:E22, TRUE)</f>
         <v>0</v>
@@ -11998,9 +10589,6 @@
       <c r="D23" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E23" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G23" s="4">
         <f>COUNTIF(B23:E23, TRUE)</f>
         <v>0</v>
@@ -12023,9 +10611,6 @@
       <c r="D24" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E24" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G24" s="4">
         <f>COUNTIF(B24:E24, TRUE)</f>
         <v>0</v>
@@ -12048,40 +10633,12 @@
       <c r="D25" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E25" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G25" s="4">
         <f>COUNTIF(B25:E25, TRUE)</f>
         <v>0</v>
       </c>
       <c r="H25" s="4">
         <f>COUNTIF(C25, TRUE)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8">
-      <c r="A26" t="s">
-        <v>41</v>
-      </c>
-      <c r="B26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="C26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="D26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="E26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="G26" s="4">
-        <f>COUNTIF(B26:E26, TRUE)</f>
-        <v>0</v>
-      </c>
-      <c r="H26" s="4">
-        <f>COUNTIF(C26, TRUE)</f>
         <v>0</v>
       </c>
     </row>
@@ -12092,7 +10649,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.140625" customWidth="1"/>
@@ -12105,25 +10662,25 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>48</v>
-      </c>
       <c r="G1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -12139,9 +10696,6 @@
       <c r="D2" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E2" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G2" s="4">
         <f>COUNTIF(B2:E2, TRUE)</f>
         <v>0</v>
@@ -12164,9 +10718,6 @@
       <c r="D3" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E3" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G3" s="4">
         <f>COUNTIF(B3:E3, TRUE)</f>
         <v>0</v>
@@ -12189,9 +10740,6 @@
       <c r="D4" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E4" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G4" s="4">
         <f>COUNTIF(B4:E4, TRUE)</f>
         <v>0</v>
@@ -12214,9 +10762,6 @@
       <c r="D5" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E5" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G5" s="4">
         <f>COUNTIF(B5:E5, TRUE)</f>
         <v>0</v>
@@ -12239,9 +10784,6 @@
       <c r="D6" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E6" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G6" s="4">
         <f>COUNTIF(B6:E6, TRUE)</f>
         <v>0</v>
@@ -12264,9 +10806,6 @@
       <c r="D7" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E7" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G7" s="4">
         <f>COUNTIF(B7:E7, TRUE)</f>
         <v>0</v>
@@ -12289,9 +10828,6 @@
       <c r="D8" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E8" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G8" s="4">
         <f>COUNTIF(B8:E8, TRUE)</f>
         <v>0</v>
@@ -12314,9 +10850,6 @@
       <c r="D9" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E9" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G9" s="4">
         <f>COUNTIF(B9:E9, TRUE)</f>
         <v>0</v>
@@ -12339,9 +10872,6 @@
       <c r="D10" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E10" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G10" s="4">
         <f>COUNTIF(B10:E10, TRUE)</f>
         <v>0</v>
@@ -12364,9 +10894,6 @@
       <c r="D11" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E11" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G11" s="4">
         <f>COUNTIF(B11:E11, TRUE)</f>
         <v>0</v>
@@ -12389,9 +10916,6 @@
       <c r="D12" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E12" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G12" s="4">
         <f>COUNTIF(B12:E12, TRUE)</f>
         <v>0</v>
@@ -12414,9 +10938,6 @@
       <c r="D13" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E13" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G13" s="4">
         <f>COUNTIF(B13:E13, TRUE)</f>
         <v>0</v>
@@ -12439,9 +10960,6 @@
       <c r="D14" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E14" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G14" s="4">
         <f>COUNTIF(B14:E14, TRUE)</f>
         <v>0</v>
@@ -12464,9 +10982,6 @@
       <c r="D15" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E15" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G15" s="4">
         <f>COUNTIF(B15:E15, TRUE)</f>
         <v>0</v>
@@ -12489,9 +11004,6 @@
       <c r="D16" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E16" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G16" s="4">
         <f>COUNTIF(B16:E16, TRUE)</f>
         <v>0</v>
@@ -12514,9 +11026,6 @@
       <c r="D17" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E17" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G17" s="4">
         <f>COUNTIF(B17:E17, TRUE)</f>
         <v>0</v>
@@ -12539,9 +11048,6 @@
       <c r="D18" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E18" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G18" s="4">
         <f>COUNTIF(B18:E18, TRUE)</f>
         <v>0</v>
@@ -12564,9 +11070,6 @@
       <c r="D19" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E19" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G19" s="4">
         <f>COUNTIF(B19:E19, TRUE)</f>
         <v>0</v>
@@ -12589,9 +11092,6 @@
       <c r="D20" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E20" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G20" s="4">
         <f>COUNTIF(B20:E20, TRUE)</f>
         <v>0</v>
@@ -12614,9 +11114,6 @@
       <c r="D21" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E21" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G21" s="4">
         <f>COUNTIF(B21:E21, TRUE)</f>
         <v>0</v>
@@ -12639,9 +11136,6 @@
       <c r="D22" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E22" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G22" s="4">
         <f>COUNTIF(B22:E22, TRUE)</f>
         <v>0</v>
@@ -12664,9 +11158,6 @@
       <c r="D23" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E23" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G23" s="4">
         <f>COUNTIF(B23:E23, TRUE)</f>
         <v>0</v>
@@ -12689,9 +11180,6 @@
       <c r="D24" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E24" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G24" s="4">
         <f>COUNTIF(B24:E24, TRUE)</f>
         <v>0</v>
@@ -12714,40 +11202,12 @@
       <c r="D25" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="E25" s="3" t="b">
-        <v>0</v>
-      </c>
       <c r="G25" s="4">
         <f>COUNTIF(B25:E25, TRUE)</f>
         <v>0</v>
       </c>
       <c r="H25" s="4">
         <f>COUNTIF(C25, TRUE)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8">
-      <c r="A26" t="s">
-        <v>41</v>
-      </c>
-      <c r="B26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="C26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="D26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="E26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="G26" s="4">
-        <f>COUNTIF(B26:E26, TRUE)</f>
-        <v>0</v>
-      </c>
-      <c r="H26" s="4">
-        <f>COUNTIF(C26, TRUE)</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
ta feature fully implemented and add_student/ remove_student bugs addressed and hopefully/ fixed.
</commit_message>
<xml_diff>
--- a/Attendance Tabloid.xlsx
+++ b/Attendance Tabloid.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="550" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="533" uniqueCount="50">
   <si>
     <t>Name</t>
   </si>
@@ -99,9 +99,6 @@
   </si>
   <si>
     <t>Brown, Trinity</t>
-  </si>
-  <si>
-    <t>Butler, Malachi</t>
   </si>
   <si>
     <t>Cranor, Christian</t>
@@ -218,7 +215,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFD9EAD3"/>
+        <fgColor rgb="FFC9DAF8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -611,7 +608,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q26"/>
+  <dimension ref="A1:Q25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="26.7109375" customWidth="1"/>
@@ -2328,77 +2325,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:17">
-      <c r="A26" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="B26" s="2">
-        <f>'Week 1'!G26</f>
-        <v>0</v>
-      </c>
-      <c r="C26" s="2">
-        <f>'Week 2'!G26</f>
-        <v>0</v>
-      </c>
-      <c r="D26" s="2">
-        <f>'Week 3'!G26</f>
-        <v>0</v>
-      </c>
-      <c r="E26" s="2">
-        <f>'Week 4'!G26</f>
-        <v>0</v>
-      </c>
-      <c r="F26" s="2">
-        <f>'Week 5'!G26</f>
-        <v>0</v>
-      </c>
-      <c r="G26" s="2">
-        <f>'Week 6'!G26</f>
-        <v>0</v>
-      </c>
-      <c r="H26" s="2">
-        <f>'Week 7'!G26</f>
-        <v>0</v>
-      </c>
-      <c r="I26" s="2">
-        <f>'Week 8'!G26</f>
-        <v>0</v>
-      </c>
-      <c r="J26" s="2">
-        <f>'Week 9'!G26</f>
-        <v>0</v>
-      </c>
-      <c r="K26" s="2">
-        <f>'Week 10'!G26</f>
-        <v>0</v>
-      </c>
-      <c r="L26" s="2">
-        <f>'Week 11'!G26</f>
-        <v>0</v>
-      </c>
-      <c r="M26" s="2">
-        <f>'Week 12'!G26</f>
-        <v>0</v>
-      </c>
-      <c r="N26" s="2">
-        <f>'Week 13'!G26</f>
-        <v>0</v>
-      </c>
-      <c r="O26" s="2">
-        <f>'Week 14'!G26</f>
-        <v>0</v>
-      </c>
-      <c r="P26" s="2">
-        <f>'Week 15'!G26</f>
-        <v>0</v>
-      </c>
-      <c r="Q26" s="2">
-        <f>SUM(B26:P26)</f>
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:P26">
+  <conditionalFormatting sqref="B2:P25">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>0</formula>
     </cfRule>
@@ -2419,7 +2347,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.140625" customWidth="1"/>
@@ -2432,25 +2360,25 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>48</v>
-      </c>
       <c r="G1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -3050,31 +2978,6 @@
       </c>
       <c r="H25" s="4">
         <f>COUNTIF(C25, TRUE)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8">
-      <c r="A26" t="s">
-        <v>41</v>
-      </c>
-      <c r="B26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="C26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="D26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="E26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="G26" s="4">
-        <f>COUNTIF(B26:E26, TRUE)</f>
-        <v>0</v>
-      </c>
-      <c r="H26" s="4">
-        <f>COUNTIF(C26, TRUE)</f>
         <v>0</v>
       </c>
     </row>
@@ -3085,7 +2988,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.140625" customWidth="1"/>
@@ -3098,25 +3001,25 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>48</v>
-      </c>
       <c r="G1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -3716,31 +3619,6 @@
       </c>
       <c r="H25" s="4">
         <f>COUNTIF(C25, TRUE)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8">
-      <c r="A26" t="s">
-        <v>41</v>
-      </c>
-      <c r="B26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="C26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="D26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="E26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="G26" s="4">
-        <f>COUNTIF(B26:E26, TRUE)</f>
-        <v>0</v>
-      </c>
-      <c r="H26" s="4">
-        <f>COUNTIF(C26, TRUE)</f>
         <v>0</v>
       </c>
     </row>
@@ -3751,7 +3629,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.140625" customWidth="1"/>
@@ -3764,25 +3642,25 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>48</v>
-      </c>
       <c r="G1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -4382,31 +4260,6 @@
       </c>
       <c r="H25" s="4">
         <f>COUNTIF(C25, TRUE)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8">
-      <c r="A26" t="s">
-        <v>41</v>
-      </c>
-      <c r="B26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="C26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="D26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="E26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="G26" s="4">
-        <f>COUNTIF(B26:E26, TRUE)</f>
-        <v>0</v>
-      </c>
-      <c r="H26" s="4">
-        <f>COUNTIF(C26, TRUE)</f>
         <v>0</v>
       </c>
     </row>
@@ -4417,7 +4270,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.140625" customWidth="1"/>
@@ -4430,25 +4283,25 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>48</v>
-      </c>
       <c r="G1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -5048,31 +4901,6 @@
       </c>
       <c r="H25" s="4">
         <f>COUNTIF(C25, TRUE)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8">
-      <c r="A26" t="s">
-        <v>41</v>
-      </c>
-      <c r="B26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="C26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="D26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="E26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="G26" s="4">
-        <f>COUNTIF(B26:E26, TRUE)</f>
-        <v>0</v>
-      </c>
-      <c r="H26" s="4">
-        <f>COUNTIF(C26, TRUE)</f>
         <v>0</v>
       </c>
     </row>
@@ -5083,7 +4911,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.140625" customWidth="1"/>
@@ -5096,25 +4924,25 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>48</v>
-      </c>
       <c r="G1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -5714,31 +5542,6 @@
       </c>
       <c r="H25" s="4">
         <f>COUNTIF(C25, TRUE)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8">
-      <c r="A26" t="s">
-        <v>41</v>
-      </c>
-      <c r="B26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="C26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="D26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="E26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="G26" s="4">
-        <f>COUNTIF(B26:E26, TRUE)</f>
-        <v>0</v>
-      </c>
-      <c r="H26" s="4">
-        <f>COUNTIF(C26, TRUE)</f>
         <v>0</v>
       </c>
     </row>
@@ -5749,7 +5552,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.140625" customWidth="1"/>
@@ -5762,25 +5565,25 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>48</v>
-      </c>
       <c r="G1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -6380,31 +6183,6 @@
       </c>
       <c r="H25" s="4">
         <f>COUNTIF(C25, TRUE)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8">
-      <c r="A26" t="s">
-        <v>41</v>
-      </c>
-      <c r="B26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="C26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="D26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="E26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="G26" s="4">
-        <f>COUNTIF(B26:E26, TRUE)</f>
-        <v>0</v>
-      </c>
-      <c r="H26" s="4">
-        <f>COUNTIF(C26, TRUE)</f>
         <v>0</v>
       </c>
     </row>
@@ -6415,7 +6193,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.140625" customWidth="1"/>
@@ -6428,25 +6206,25 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>48</v>
-      </c>
       <c r="G1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -7046,31 +6824,6 @@
       </c>
       <c r="H25" s="4">
         <f>COUNTIF(C25, TRUE)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8">
-      <c r="A26" t="s">
-        <v>41</v>
-      </c>
-      <c r="B26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="C26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="D26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="E26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="G26" s="4">
-        <f>COUNTIF(B26:E26, TRUE)</f>
-        <v>0</v>
-      </c>
-      <c r="H26" s="4">
-        <f>COUNTIF(C26, TRUE)</f>
         <v>0</v>
       </c>
     </row>
@@ -7081,7 +6834,7 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="26.7109375" customWidth="1"/>
@@ -7089,13 +6842,13 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -7407,19 +7160,6 @@
       </c>
       <c r="C25" s="5">
         <f>SUM('Week 1:Week 15'!H25) / 16</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3">
-      <c r="A26" t="s">
-        <v>41</v>
-      </c>
-      <c r="B26" s="4">
-        <f>SUM('Week 1:Week 15'!H26)</f>
-        <v>0</v>
-      </c>
-      <c r="C26" s="5">
-        <f>SUM('Week 1:Week 15'!H26) / 16</f>
         <v>0</v>
       </c>
     </row>
@@ -7430,7 +7170,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.140625" customWidth="1"/>
@@ -7443,25 +7183,25 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>48</v>
-      </c>
       <c r="G1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -7519,7 +7259,7 @@
         <v>19</v>
       </c>
       <c r="B4" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C4" s="3" t="b">
         <v>0</v>
@@ -7544,7 +7284,7 @@
         <v>20</v>
       </c>
       <c r="B5" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C5" s="3" t="b">
         <v>0</v>
@@ -7569,7 +7309,7 @@
         <v>21</v>
       </c>
       <c r="B6" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C6" s="3" t="b">
         <v>0</v>
@@ -7594,7 +7334,7 @@
         <v>22</v>
       </c>
       <c r="B7" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C7" s="3" t="b">
         <v>0</v>
@@ -7619,7 +7359,7 @@
         <v>23</v>
       </c>
       <c r="B8" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C8" s="3" t="b">
         <v>0</v>
@@ -8061,31 +7801,6 @@
       </c>
       <c r="H25" s="4">
         <f>COUNTIF(C25, TRUE)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8">
-      <c r="A26" t="s">
-        <v>41</v>
-      </c>
-      <c r="B26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="C26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="D26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="E26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="G26" s="4">
-        <f>COUNTIF(B26:E26, TRUE)</f>
-        <v>0</v>
-      </c>
-      <c r="H26" s="4">
-        <f>COUNTIF(C26, TRUE)</f>
         <v>0</v>
       </c>
     </row>
@@ -8096,7 +7811,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.140625" customWidth="1"/>
@@ -8109,25 +7824,25 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>48</v>
-      </c>
       <c r="G1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -8727,31 +8442,6 @@
       </c>
       <c r="H25" s="4">
         <f>COUNTIF(C25, TRUE)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8">
-      <c r="A26" t="s">
-        <v>41</v>
-      </c>
-      <c r="B26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="C26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="D26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="E26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="G26" s="4">
-        <f>COUNTIF(B26:E26, TRUE)</f>
-        <v>0</v>
-      </c>
-      <c r="H26" s="4">
-        <f>COUNTIF(C26, TRUE)</f>
         <v>0</v>
       </c>
     </row>
@@ -8762,7 +8452,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.140625" customWidth="1"/>
@@ -8775,25 +8465,25 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>48</v>
-      </c>
       <c r="G1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -9393,31 +9083,6 @@
       </c>
       <c r="H25" s="4">
         <f>COUNTIF(C25, TRUE)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8">
-      <c r="A26" t="s">
-        <v>41</v>
-      </c>
-      <c r="B26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="C26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="D26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="E26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="G26" s="4">
-        <f>COUNTIF(B26:E26, TRUE)</f>
-        <v>0</v>
-      </c>
-      <c r="H26" s="4">
-        <f>COUNTIF(C26, TRUE)</f>
         <v>0</v>
       </c>
     </row>
@@ -9428,7 +9093,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.140625" customWidth="1"/>
@@ -9441,25 +9106,25 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>48</v>
-      </c>
       <c r="G1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -10059,31 +9724,6 @@
       </c>
       <c r="H25" s="4">
         <f>COUNTIF(C25, TRUE)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8">
-      <c r="A26" t="s">
-        <v>41</v>
-      </c>
-      <c r="B26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="C26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="D26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="E26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="G26" s="4">
-        <f>COUNTIF(B26:E26, TRUE)</f>
-        <v>0</v>
-      </c>
-      <c r="H26" s="4">
-        <f>COUNTIF(C26, TRUE)</f>
         <v>0</v>
       </c>
     </row>
@@ -10094,7 +9734,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.140625" customWidth="1"/>
@@ -10107,25 +9747,25 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>48</v>
-      </c>
       <c r="G1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -10725,31 +10365,6 @@
       </c>
       <c r="H25" s="4">
         <f>COUNTIF(C25, TRUE)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8">
-      <c r="A26" t="s">
-        <v>41</v>
-      </c>
-      <c r="B26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="C26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="D26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="E26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="G26" s="4">
-        <f>COUNTIF(B26:E26, TRUE)</f>
-        <v>0</v>
-      </c>
-      <c r="H26" s="4">
-        <f>COUNTIF(C26, TRUE)</f>
         <v>0</v>
       </c>
     </row>
@@ -10760,7 +10375,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.140625" customWidth="1"/>
@@ -10773,25 +10388,25 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>48</v>
-      </c>
       <c r="G1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -11391,31 +11006,6 @@
       </c>
       <c r="H25" s="4">
         <f>COUNTIF(C25, TRUE)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8">
-      <c r="A26" t="s">
-        <v>41</v>
-      </c>
-      <c r="B26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="C26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="D26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="E26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="G26" s="4">
-        <f>COUNTIF(B26:E26, TRUE)</f>
-        <v>0</v>
-      </c>
-      <c r="H26" s="4">
-        <f>COUNTIF(C26, TRUE)</f>
         <v>0</v>
       </c>
     </row>
@@ -11426,7 +11016,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.140625" customWidth="1"/>
@@ -11439,25 +11029,25 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>48</v>
-      </c>
       <c r="G1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -12057,31 +11647,6 @@
       </c>
       <c r="H25" s="4">
         <f>COUNTIF(C25, TRUE)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8">
-      <c r="A26" t="s">
-        <v>41</v>
-      </c>
-      <c r="B26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="C26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="D26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="E26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="G26" s="4">
-        <f>COUNTIF(B26:E26, TRUE)</f>
-        <v>0</v>
-      </c>
-      <c r="H26" s="4">
-        <f>COUNTIF(C26, TRUE)</f>
         <v>0</v>
       </c>
     </row>
@@ -12092,7 +11657,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.140625" customWidth="1"/>
@@ -12105,25 +11670,25 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>48</v>
-      </c>
       <c r="G1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -12723,31 +12288,6 @@
       </c>
       <c r="H25" s="4">
         <f>COUNTIF(C25, TRUE)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8">
-      <c r="A26" t="s">
-        <v>41</v>
-      </c>
-      <c r="B26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="C26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="D26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="E26" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="G26" s="4">
-        <f>COUNTIF(B26:E26, TRUE)</f>
-        <v>0</v>
-      </c>
-      <c r="H26" s="4">
-        <f>COUNTIF(C26, TRUE)</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>